<commit_message>
Update database of standard entropy of compounds
</commit_message>
<xml_diff>
--- a/ecosysem/db/Excels/S0.xlsx
+++ b/ecosysem/db/Excels/S0.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emartinez\Documents\GitHub\EcoSysEM\ecosysem\db\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B288C6-8E31-442B-A254-FA4FD3624AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D19C4B9D-D8C9-4691-A3A3-4B50081A8632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5025" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{B28E7694-DBED-47BF-AE0C-82F612E0B7E3}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{B28E7694-DBED-47BF-AE0C-82F612E0B7E3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="S0" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +58,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    [J/mo/Kl]</t>
+    [J/mol/K]</t>
       </text>
     </comment>
   </commentList>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
   <si>
     <t>IUPAC</t>
   </si>
@@ -159,13 +159,61 @@
   </si>
   <si>
     <t>Asm.</t>
+  </si>
+  <si>
+    <t>Bicarbonate</t>
+  </si>
+  <si>
+    <t>HCO3-</t>
+  </si>
+  <si>
+    <t>Carbonate</t>
+  </si>
+  <si>
+    <t>CO3-2</t>
+  </si>
+  <si>
+    <t>Ammonium</t>
+  </si>
+  <si>
+    <t>NH4+</t>
+  </si>
+  <si>
+    <t>Nitrous acid</t>
+  </si>
+  <si>
+    <t>HNO2</t>
+  </si>
+  <si>
+    <t>Bisulfide</t>
+  </si>
+  <si>
+    <t>HS-</t>
+  </si>
+  <si>
+    <t>Sulfide</t>
+  </si>
+  <si>
+    <t>S-2</t>
+  </si>
+  <si>
+    <t>Sulfuric acid</t>
+  </si>
+  <si>
+    <t>H2SO4</t>
+  </si>
+  <si>
+    <t>Hydrogen sulfate</t>
+  </si>
+  <si>
+    <t>HSO4-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,12 +228,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
@@ -216,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -225,10 +267,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -576,14 +615,14 @@
     <text>'aq' as 'L'</text>
   </threadedComment>
   <threadedComment ref="D1" dT="2026-04-29T20:01:23.77" personId="{4A5AEA47-CF44-4814-94FC-A1AAC57893C4}" id="{BA3A7C06-B1F1-45C8-8E7D-E4793AC3F190}">
-    <text>[J/mo/Kl]</text>
+    <text>[J/mol/K]</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2A0639D-45DA-4D3C-9ECA-52A3EC242CC4}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -617,7 +656,7 @@
       <c r="B2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="3">
@@ -634,7 +673,7 @@
       <c r="B3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="3">
@@ -651,7 +690,7 @@
       <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="3">
@@ -668,7 +707,7 @@
       <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="3">
@@ -685,7 +724,7 @@
       <c r="B6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="3">
@@ -697,16 +736,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="3">
-        <v>69.95</v>
+        <v>98.45</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>22</v>
@@ -714,16 +753,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>17</v>
+        <v>34</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D8" s="3">
-        <v>130.68</v>
+        <v>-50.01</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>22</v>
@@ -731,103 +770,103 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="3">
-        <v>130.68</v>
+        <v>69.95</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="3">
-        <v>119.66</v>
+        <v>130.68</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="3">
-        <v>119.66</v>
+        <v>130.68</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12" s="3">
-        <v>126.5</v>
+        <v>119.66</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>22</v>
       </c>
+      <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="3">
-        <v>18.5</v>
+        <v>119.66</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D14" s="3">
-        <v>0</v>
+        <v>126.5</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>22</v>
@@ -835,16 +874,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D15" s="3">
-        <v>111.3</v>
+        <v>67.5</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>22</v>
@@ -852,18 +891,188 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="3">
+        <v>22</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="3">
+        <v>156.9</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="3">
+        <v>131.72999999999999</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="3">
+        <v>18.5</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="3">
+        <v>192.77600000000001</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="3">
+        <v>111.3</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="3">
+        <v>111.17</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="3">
+        <v>254.1</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="3">
+        <v>254.1</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="3">
+      <c r="C26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="3">
         <v>123</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>